<commit_message>
fix(warehouse): make DO number formatting conditional on BOX items
</commit_message>
<xml_diff>
--- a/public/assets/Master List Aset bubblesO2.xlsx
+++ b/public/assets/Master List Aset bubblesO2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Aset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\All in One System\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3E043B-BA8C-47F2-98A9-DFA0A46CE031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B28686D-CAD6-4184-B793-998E32F94902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{45242A28-43C0-4D13-83D7-864AFD64D9CF}"/>
   </bookViews>
@@ -2615,6 +2615,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FBE5F04-AE9B-43AD-AF7F-B7067EF91388}">
   <dimension ref="A1:BC314"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="12" max="12" width="19.33203125" customWidth="1"/>
+    <col min="28" max="28" width="20.33203125" customWidth="1"/>
+    <col min="31" max="32" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="14.44140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
style(pmr): enlarge text size and improve table visibility for SGMP-03 PMR report
</commit_message>
<xml_diff>
--- a/public/assets/Master List Aset bubblesO2.xlsx
+++ b/public/assets/Master List Aset bubblesO2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\All in One System\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B28686D-CAD6-4184-B793-998E32F94902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF1F7AE-AA9A-4D03-B404-253487770292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{45242A28-43C0-4D13-83D7-864AFD64D9CF}"/>
   </bookViews>
@@ -2619,6 +2619,7 @@
     <col min="12" max="12" width="19.33203125" customWidth="1"/>
     <col min="28" max="28" width="20.33203125" customWidth="1"/>
     <col min="31" max="32" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="46.21875" customWidth="1"/>
     <col min="49" max="49" width="14.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>